<commit_message>
Fix welfare preprocessing with scoped three-valued conditions and preserve unknown requirements
</commit_message>
<xml_diff>
--- a/tables/analysis_tables.xlsx
+++ b/tables/analysis_tables.xlsx
@@ -542,7 +542,7 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>이용 희망 전제의 기본 안내; 실제 자격 확정 아님</t>
+          <t>v3 관측조건·일반안내. 미관측 상담·교육 필요성은미확인; 실제 자격 확정 아님</t>
         </is>
       </c>
     </row>
@@ -574,17 +574,17 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>법률상담을 원하는 국민</t>
+          <t>법률상담이 필요한 국민</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>현재국적코드=1: 기본 안내; 그 외 미확인</t>
+          <t>국적은 관측; 상담 필요성은 미확인</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>이용 희망 전제의 기본 안내; 실제 자격 확정 아님</t>
+          <t>v3 관측조건·일반안내. 미관측 상담·교육 필요성은미확인; 실제 자격 확정 아님</t>
         </is>
       </c>
     </row>
@@ -626,7 +626,7 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>이용 희망 전제의 기본 안내; 실제 자격 확정 아님</t>
+          <t>v3 관측조건·일반안내. 미관측 상담·교육 필요성은미확인; 실제 자격 확정 아님</t>
         </is>
       </c>
     </row>
@@ -658,17 +658,17 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>일반 국민 대상 성교육 서비스</t>
+          <t>아동청소년·교사·양육자 등 대상별 성교육</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>현재국적코드=1: 기본 안내; 그 외 미확인</t>
+          <t>개별 프로그램 대상 범위가 미확정이므로 미확인</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>이용 희망 전제의 기본 안내; 실제 자격 확정 아님</t>
+          <t>v3 관측조건·일반안내. 미관측 상담·교육 필요성은미확인; 실제 자격 확정 아님</t>
         </is>
       </c>
     </row>
@@ -710,7 +710,7 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>이용 희망 전제의 기본 안내; 실제 자격 확정 아님</t>
+          <t>v3 관측조건·일반안내. 미관측 상담·교육 필요성은미확인; 실제 자격 확정 아님</t>
         </is>
       </c>
     </row>
@@ -742,17 +742,17 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>디지털 교육을 원하는 국민</t>
+          <t>AI·디지털에 어려움을 겪는 국민</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>현재국적코드=1: 기본 안내; 그 외 미확인</t>
+          <t>디지털 어려움은 미관측이므로 미확인</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>이용 희망 전제의 기본 안내; 실제 자격 확정 아님</t>
+          <t>v3 관측조건·일반안내. 미관측 상담·교육 필요성은미확인; 실제 자격 확정 아님</t>
         </is>
       </c>
     </row>
@@ -784,17 +784,17 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>정보화교육을 원하는 장애인</t>
+          <t>정보화교육이 필요한 장애인</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>장애인복지카드_소유여부=1: 기본 안내; 미소유/결측은 미확인</t>
+          <t>등록상태·교육 필요성은 미확인; 카드 미소유로 비장애 추정 금지</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>이용 희망 전제의 기본 안내; 실제 자격 확정 아님</t>
+          <t>v3 관측조건·일반안내. 미관측 상담·교육 필요성은미확인; 실제 자격 확정 아님</t>
         </is>
       </c>
     </row>
@@ -826,17 +826,17 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>초·중·고 재학생의 일반 상담</t>
+          <t>초·중·고 재학생 중 상담·교육활동이 필요한 학생</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>교육정도코드∈{1,2,3} AND 재학상태코드=3; 결측 보존</t>
+          <t>초중고 재학 AND 상담 필요성(미관측); 미재학생은 관측조건 비해당</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>이용 희망 전제의 기본 안내; 실제 자격 확정 아님</t>
+          <t>v3 관측조건·일반안내. 미관측 상담·교육 필요성은미확인; 실제 자격 확정 아님</t>
         </is>
       </c>
     </row>
@@ -1179,10 +1179,10 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>33388</v>
+        <v>0</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>97.96404572124085</v>
+        <v>0</v>
       </c>
       <c r="E3" s="2" t="n">
         <v>0</v>
@@ -1191,10 +1191,10 @@
         <v>0</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>556</v>
+        <v>33944</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>2.035954278759167</v>
+        <v>100</v>
       </c>
     </row>
     <row r="4" ht="46" customHeight="1">
@@ -1239,10 +1239,10 @@
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>33388</v>
+        <v>0</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>97.96404572124085</v>
+        <v>0</v>
       </c>
       <c r="E5" s="2" t="n">
         <v>0</v>
@@ -1251,10 +1251,10 @@
         <v>0</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>556</v>
+        <v>33944</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>2.035954278759167</v>
+        <v>100</v>
       </c>
     </row>
     <row r="6" ht="46" customHeight="1">
@@ -1299,10 +1299,10 @@
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>33388</v>
+        <v>0</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>97.96404572124085</v>
+        <v>0</v>
       </c>
       <c r="E7" s="2" t="n">
         <v>0</v>
@@ -1311,10 +1311,10 @@
         <v>0</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>556</v>
+        <v>33944</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>2.035954278759167</v>
+        <v>100</v>
       </c>
     </row>
     <row r="8" ht="46" customHeight="1">
@@ -1329,10 +1329,10 @@
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>2052</v>
+        <v>0</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>4.851506976765293</v>
+        <v>0</v>
       </c>
       <c r="E8" s="2" t="n">
         <v>0</v>
@@ -1341,10 +1341,10 @@
         <v>0</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>31892</v>
+        <v>33944</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>95.14849302323471</v>
+        <v>100</v>
       </c>
     </row>
     <row r="9" ht="46" customHeight="1">
@@ -1359,10 +1359,10 @@
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>1707</v>
+        <v>0</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>5.405784963094085</v>
+        <v>0</v>
       </c>
       <c r="E9" s="2" t="n">
         <v>32237</v>
@@ -1371,10 +1371,10 @@
         <v>94.59421503690592</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>0</v>
+        <v>1707</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>0</v>
+        <v>5.405784963094085</v>
       </c>
     </row>
   </sheetData>
@@ -1442,16 +1442,16 @@
         <v>1884</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>6.887041660648552</v>
+        <v>2.99391874770756</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>1.016410371149326</v>
+        <v>4.909533284090318</v>
       </c>
       <c r="E2" s="2" t="n">
         <v>0.09654796820212168</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3" ht="46" customHeight="1">
@@ -1464,16 +1464,16 @@
         <v>5393</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>5.864923456518604</v>
+        <v>2.962221259765975</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>1.1352231093131</v>
+        <v>4.03792530606573</v>
       </c>
       <c r="E3" s="2" t="n">
         <v>0.9998534341682955</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4" ht="46" customHeight="1">
@@ -1486,16 +1486,16 @@
         <v>17171</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>5.954254136142636</v>
+        <v>2.980010818731821</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>1.045745863857363</v>
+        <v>4.019989181268179</v>
       </c>
       <c r="E4" s="2" t="n">
         <v>1</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5" ht="46" customHeight="1">
@@ -1508,16 +1508,16 @@
         <v>9496</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>6.094833833273327</v>
+        <v>2.992154697647897</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>0.9052098653841553</v>
+        <v>4.007889001009585</v>
       </c>
       <c r="E5" s="2" t="n">
         <v>0.9999563013425184</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -1585,16 +1585,16 @@
         <v>31892</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>5.970826565393924</v>
+        <v>2.978621544606899</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>1.085513821572407</v>
+        <v>4.077718842359433</v>
       </c>
       <c r="E2" s="2" t="n">
         <v>0.9436596130336702</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3" ht="46" customHeight="1">
@@ -1607,16 +1607,16 @@
         <v>2052</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>7.007786485172222</v>
+        <v>2.999623526267231</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>0.001505894931074668</v>
+        <v>4.009668853836065</v>
       </c>
       <c r="E3" s="2" t="n">
         <v>0.9907076198967031</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>